<commit_message>
Feature - processamento geral utilizando a sintaxe
</commit_message>
<xml_diff>
--- a/Sintaxe_Exemplo.xlsx
+++ b/Sintaxe_Exemplo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJETOS\Processamento-Estatistico\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJETOS\Expertise\Processamento-Estatistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40180706-A58D-49F5-9108-D55ADEB23E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFBBBC2-A896-47B7-A88F-BEBAD2AA76A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1026,6 +1026,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="G5" twoDigitTextYear="1"/>
+  </ignoredErrors>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>